<commit_message>
update temp data and graphs
</commit_message>
<xml_diff>
--- a/Behavioral figures/Male cohort 2 - PO/Data to plot - cohort 2.xlsx
+++ b/Behavioral figures/Male cohort 2 - PO/Data to plot - cohort 2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mchakra/Dropbox/Stanford/Research/Bhatt lab/Computation/BBB project/Paper code/Behavioral figures/Male cohort 2 - PO/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF1C0E58-05EE-DB44-8618-3828D16011B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC1A7EC-4A80-5E41-BB64-3B5F5EDF574A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1580" yWindow="600" windowWidth="18380" windowHeight="19260" activeTab="1" xr2:uid="{B97866B8-D1E9-AE49-A867-7C16CE79F6E8}"/>
+    <workbookView xWindow="1580" yWindow="600" windowWidth="21900" windowHeight="22880" activeTab="1" xr2:uid="{B97866B8-D1E9-AE49-A867-7C16CE79F6E8}"/>
   </bookViews>
   <sheets>
     <sheet name="Ymaze_2" sheetId="4" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1089" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1134" uniqueCount="21">
   <si>
     <t>Mouse ID</t>
   </si>
@@ -97,6 +97,9 @@
   </si>
   <si>
     <t>Time</t>
+  </si>
+  <si>
+    <t>Baseline</t>
   </si>
 </sst>
 </file>
@@ -7779,8 +7782,8 @@
       <c r="B2" t="s">
         <v>4</v>
       </c>
-      <c r="C2">
-        <v>0</v>
+      <c r="C2" t="s">
+        <v>20</v>
       </c>
       <c r="D2">
         <v>37.9</v>
@@ -7793,8 +7796,8 @@
       <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="C3">
-        <v>0</v>
+      <c r="C3" t="s">
+        <v>20</v>
       </c>
       <c r="D3">
         <v>38.4</v>
@@ -7807,8 +7810,8 @@
       <c r="B4" t="s">
         <v>4</v>
       </c>
-      <c r="C4">
-        <v>0</v>
+      <c r="C4" t="s">
+        <v>20</v>
       </c>
       <c r="D4">
         <v>38.200000000000003</v>
@@ -7821,8 +7824,8 @@
       <c r="B5" t="s">
         <v>4</v>
       </c>
-      <c r="C5">
-        <v>0</v>
+      <c r="C5" t="s">
+        <v>20</v>
       </c>
       <c r="D5">
         <v>38.200000000000003</v>
@@ -7835,8 +7838,8 @@
       <c r="B6" t="s">
         <v>4</v>
       </c>
-      <c r="C6">
-        <v>0</v>
+      <c r="C6" t="s">
+        <v>20</v>
       </c>
       <c r="D6">
         <v>38.1</v>
@@ -7849,8 +7852,8 @@
       <c r="B7" t="s">
         <v>4</v>
       </c>
-      <c r="C7">
-        <v>0</v>
+      <c r="C7" t="s">
+        <v>20</v>
       </c>
       <c r="D7">
         <v>38.200000000000003</v>
@@ -7863,8 +7866,8 @@
       <c r="B8" t="s">
         <v>4</v>
       </c>
-      <c r="C8">
-        <v>0</v>
+      <c r="C8" t="s">
+        <v>20</v>
       </c>
       <c r="D8">
         <v>38.4</v>
@@ -7877,8 +7880,8 @@
       <c r="B9" t="s">
         <v>4</v>
       </c>
-      <c r="C9">
-        <v>0</v>
+      <c r="C9" t="s">
+        <v>20</v>
       </c>
       <c r="D9">
         <v>38</v>
@@ -7891,8 +7894,8 @@
       <c r="B10" t="s">
         <v>4</v>
       </c>
-      <c r="C10">
-        <v>0</v>
+      <c r="C10" t="s">
+        <v>20</v>
       </c>
       <c r="D10">
         <v>38.299999999999997</v>
@@ -7905,8 +7908,8 @@
       <c r="B11" t="s">
         <v>4</v>
       </c>
-      <c r="C11">
-        <v>0</v>
+      <c r="C11" t="s">
+        <v>20</v>
       </c>
       <c r="D11">
         <v>38.700000000000003</v>
@@ -7919,8 +7922,8 @@
       <c r="B12" t="s">
         <v>4</v>
       </c>
-      <c r="C12">
-        <v>0</v>
+      <c r="C12" t="s">
+        <v>20</v>
       </c>
       <c r="D12">
         <v>36.5</v>
@@ -7933,8 +7936,8 @@
       <c r="B13" t="s">
         <v>4</v>
       </c>
-      <c r="C13">
-        <v>0</v>
+      <c r="C13" t="s">
+        <v>20</v>
       </c>
       <c r="D13">
         <v>36.799999999999997</v>
@@ -7947,8 +7950,8 @@
       <c r="B14" t="s">
         <v>4</v>
       </c>
-      <c r="C14">
-        <v>0</v>
+      <c r="C14" t="s">
+        <v>20</v>
       </c>
       <c r="D14">
         <v>36.6</v>
@@ -7961,8 +7964,8 @@
       <c r="B15" t="s">
         <v>4</v>
       </c>
-      <c r="C15">
-        <v>0</v>
+      <c r="C15" t="s">
+        <v>20</v>
       </c>
       <c r="D15">
         <v>37.200000000000003</v>
@@ -7975,8 +7978,8 @@
       <c r="B16" t="s">
         <v>4</v>
       </c>
-      <c r="C16">
-        <v>0</v>
+      <c r="C16" t="s">
+        <v>20</v>
       </c>
       <c r="D16">
         <v>36.5</v>
@@ -7989,8 +7992,8 @@
       <c r="B17" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C17">
-        <v>0</v>
+      <c r="C17" t="s">
+        <v>20</v>
       </c>
       <c r="D17">
         <v>36.299999999999997</v>
@@ -8003,8 +8006,8 @@
       <c r="B18" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C18">
-        <v>0</v>
+      <c r="C18" t="s">
+        <v>20</v>
       </c>
       <c r="D18">
         <v>37.6</v>
@@ -8017,8 +8020,8 @@
       <c r="B19" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C19">
-        <v>0</v>
+      <c r="C19" t="s">
+        <v>20</v>
       </c>
       <c r="D19">
         <v>38.1</v>
@@ -8031,8 +8034,8 @@
       <c r="B20" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C20">
-        <v>0</v>
+      <c r="C20" t="s">
+        <v>20</v>
       </c>
       <c r="D20">
         <v>37.299999999999997</v>
@@ -8045,8 +8048,8 @@
       <c r="B21" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C21">
-        <v>0</v>
+      <c r="C21" t="s">
+        <v>20</v>
       </c>
       <c r="D21">
         <v>37.9</v>
@@ -8059,8 +8062,8 @@
       <c r="B22" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C22">
-        <v>0</v>
+      <c r="C22" t="s">
+        <v>20</v>
       </c>
       <c r="D22">
         <v>36.700000000000003</v>
@@ -8073,8 +8076,8 @@
       <c r="B23" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C23">
-        <v>0</v>
+      <c r="C23" t="s">
+        <v>20</v>
       </c>
       <c r="D23">
         <v>36.799999999999997</v>
@@ -8087,8 +8090,8 @@
       <c r="B24" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C24">
-        <v>0</v>
+      <c r="C24" t="s">
+        <v>20</v>
       </c>
       <c r="D24">
         <v>36.1</v>
@@ -8101,8 +8104,8 @@
       <c r="B25" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C25">
-        <v>0</v>
+      <c r="C25" t="s">
+        <v>20</v>
       </c>
       <c r="D25">
         <v>36.4</v>
@@ -8115,8 +8118,8 @@
       <c r="B26" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C26">
-        <v>0</v>
+      <c r="C26" t="s">
+        <v>20</v>
       </c>
       <c r="D26">
         <v>37</v>
@@ -8129,8 +8132,8 @@
       <c r="B27" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C27">
-        <v>0</v>
+      <c r="C27" t="s">
+        <v>20</v>
       </c>
       <c r="D27">
         <v>36</v>
@@ -8143,8 +8146,8 @@
       <c r="B28" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C28">
-        <v>0</v>
+      <c r="C28" t="s">
+        <v>20</v>
       </c>
       <c r="D28">
         <v>36.4</v>
@@ -8157,8 +8160,8 @@
       <c r="B29" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C29">
-        <v>0</v>
+      <c r="C29" t="s">
+        <v>20</v>
       </c>
       <c r="D29">
         <v>36</v>
@@ -8171,8 +8174,8 @@
       <c r="B30" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C30">
-        <v>0</v>
+      <c r="C30" t="s">
+        <v>20</v>
       </c>
       <c r="D30">
         <v>36.700000000000003</v>
@@ -8185,8 +8188,8 @@
       <c r="B31" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C31">
-        <v>0</v>
+      <c r="C31" t="s">
+        <v>20</v>
       </c>
       <c r="D31">
         <v>36.799999999999997</v>
@@ -8199,8 +8202,8 @@
       <c r="B32" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C32">
-        <v>0</v>
+      <c r="C32" t="s">
+        <v>20</v>
       </c>
       <c r="D32">
         <v>35.799999999999997</v>
@@ -8213,8 +8216,8 @@
       <c r="B33" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C33">
-        <v>0</v>
+      <c r="C33" t="s">
+        <v>20</v>
       </c>
       <c r="D33">
         <v>36.5</v>
@@ -8227,8 +8230,8 @@
       <c r="B34" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C34">
-        <v>0</v>
+      <c r="C34" t="s">
+        <v>20</v>
       </c>
       <c r="D34">
         <v>37.200000000000003</v>
@@ -8241,8 +8244,8 @@
       <c r="B35" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C35">
-        <v>0</v>
+      <c r="C35" t="s">
+        <v>20</v>
       </c>
       <c r="D35">
         <v>37.1</v>
@@ -8255,8 +8258,8 @@
       <c r="B36" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C36">
-        <v>0</v>
+      <c r="C36" t="s">
+        <v>20</v>
       </c>
       <c r="D36">
         <v>37.200000000000003</v>
@@ -8269,8 +8272,8 @@
       <c r="B37" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C37">
-        <v>0</v>
+      <c r="C37" t="s">
+        <v>20</v>
       </c>
       <c r="D37">
         <v>36.799999999999997</v>
@@ -8283,8 +8286,8 @@
       <c r="B38" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C38">
-        <v>0</v>
+      <c r="C38" t="s">
+        <v>20</v>
       </c>
       <c r="D38">
         <v>38.1</v>
@@ -8297,8 +8300,8 @@
       <c r="B39" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C39">
-        <v>0</v>
+      <c r="C39" t="s">
+        <v>20</v>
       </c>
       <c r="D39">
         <v>37.799999999999997</v>
@@ -8311,8 +8314,8 @@
       <c r="B40" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C40">
-        <v>0</v>
+      <c r="C40" t="s">
+        <v>20</v>
       </c>
       <c r="D40">
         <v>38.299999999999997</v>
@@ -8325,8 +8328,8 @@
       <c r="B41" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C41">
-        <v>0</v>
+      <c r="C41" t="s">
+        <v>20</v>
       </c>
       <c r="D41">
         <v>37</v>
@@ -8339,8 +8342,8 @@
       <c r="B42" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C42">
-        <v>0</v>
+      <c r="C42" t="s">
+        <v>20</v>
       </c>
       <c r="D42">
         <v>36.299999999999997</v>
@@ -8353,8 +8356,8 @@
       <c r="B43" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C43">
-        <v>0</v>
+      <c r="C43" t="s">
+        <v>20</v>
       </c>
       <c r="D43">
         <v>36.4</v>
@@ -8367,8 +8370,8 @@
       <c r="B44" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C44">
-        <v>0</v>
+      <c r="C44" t="s">
+        <v>20</v>
       </c>
       <c r="D44">
         <v>36.299999999999997</v>
@@ -8381,8 +8384,8 @@
       <c r="B45" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C45">
-        <v>0</v>
+      <c r="C45" t="s">
+        <v>20</v>
       </c>
       <c r="D45">
         <v>36.4</v>
@@ -8395,8 +8398,8 @@
       <c r="B46" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C46">
-        <v>0</v>
+      <c r="C46" t="s">
+        <v>20</v>
       </c>
       <c r="D46">
         <v>37.1</v>

</xml_diff>